<commit_message>
added data from 2025, prepped it all
</commit_message>
<xml_diff>
--- a/analysis/data/raw_data/Dungeness_sppcomp_data_2024_BC.xlsx
+++ b/analysis/data/raw_data/Dungeness_sppcomp_data_2024_BC.xlsx
@@ -36735,4 +36735,10 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{45011977-b912-4387-97a4-f4c94a801377}" enabled="1" method="Standard" siteId="{11d0e217-264e-400a-8ba0-57dcc127d72d}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>